<commit_message>
Add new temperature time series data for 2026
</commit_message>
<xml_diff>
--- a/resultados_python/terreno_2026_hatch/datos_terreno/tabla_iqr_hatch_amplitude.xlsx
+++ b/resultados_python/terreno_2026_hatch/datos_terreno/tabla_iqr_hatch_amplitude.xlsx
@@ -470,19 +470,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>337.3</v>
+        <v>347.3</v>
       </c>
       <c r="C2" t="n">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D2" t="n">
-        <v>336.9</v>
+        <v>345.9</v>
       </c>
       <c r="E2" t="n">
-        <v>346.3</v>
+        <v>363.9</v>
       </c>
       <c r="F2" t="n">
-        <v>18.4</v>
+        <v>34</v>
       </c>
       <c r="G2" t="n">
         <v>3</v>
@@ -491,7 +491,7 @@
         <v>281</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="3">
@@ -501,19 +501,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>315.9</v>
+        <v>330.3</v>
       </c>
       <c r="C3" t="n">
-        <v>309.7</v>
+        <v>323</v>
       </c>
       <c r="D3" t="n">
-        <v>315.7</v>
+        <v>330</v>
       </c>
       <c r="E3" t="n">
-        <v>322.1</v>
+        <v>337.5</v>
       </c>
       <c r="F3" t="n">
-        <v>12.4</v>
+        <v>14.6</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
@@ -522,7 +522,7 @@
         <v>311</v>
       </c>
       <c r="I3" t="n">
-        <v>1.6</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="4">
@@ -532,19 +532,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>664.1</v>
+        <v>1720.1</v>
       </c>
       <c r="C4" t="n">
-        <v>608.3</v>
+        <v>1452.3</v>
       </c>
       <c r="D4" t="n">
-        <v>645.7</v>
+        <v>1622.7</v>
       </c>
       <c r="E4" t="n">
-        <v>710.6</v>
+        <v>1939.2</v>
       </c>
       <c r="F4" t="n">
-        <v>103.6</v>
+        <v>494.1</v>
       </c>
       <c r="G4" t="n">
         <v>3</v>
@@ -553,7 +553,7 @@
         <v>2246</v>
       </c>
       <c r="I4" t="n">
-        <v>-70.40000000000001</v>
+        <v>-23.4</v>
       </c>
     </row>
     <row r="5">
@@ -563,19 +563,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>677.8</v>
+        <v>1739.5</v>
       </c>
       <c r="C5" t="n">
-        <v>665.4</v>
+        <v>1675.3</v>
       </c>
       <c r="D5" t="n">
-        <v>676.8</v>
+        <v>1733.5</v>
       </c>
       <c r="E5" t="n">
-        <v>689.7</v>
+        <v>1800.8</v>
       </c>
       <c r="F5" t="n">
-        <v>24.3</v>
+        <v>125.6</v>
       </c>
       <c r="G5" t="n">
         <v>3</v>
@@ -584,7 +584,7 @@
         <v>1555</v>
       </c>
       <c r="I5" t="n">
-        <v>-56.4</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="6">
@@ -594,19 +594,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>220.3</v>
+        <v>220</v>
       </c>
       <c r="C6" t="n">
-        <v>173.4</v>
+        <v>157.2</v>
       </c>
       <c r="D6" t="n">
-        <v>211.8</v>
+        <v>200.7</v>
       </c>
       <c r="E6" t="n">
-        <v>262.9</v>
+        <v>273.2</v>
       </c>
       <c r="F6" t="n">
-        <v>89.8</v>
+        <v>117.2</v>
       </c>
       <c r="G6" t="n">
         <v>3</v>
@@ -615,7 +615,7 @@
         <v>181</v>
       </c>
       <c r="I6" t="n">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>